<commit_message>
test(examples): 以0.2.0构建器重建样例并更新验收日志(Checks 12/12 ALL PASS)
</commit_message>
<xml_diff>
--- a/examples/002463_沪电股份_估值模型.xlsx
+++ b/examples/002463_沪电股份_估值模型.xlsx
@@ -19,12 +19,29 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FIN" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equity_Roll" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relative_Val" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenarios" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FCFE" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relative_Val" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenarios" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="SCEN_SWITCH">Assumptions!$C$5</definedName>
+    <definedName name="WACC_USED">Assumptions!$C$86</definedName>
+    <definedName name="WACC_CALC">Assumptions!$C$84</definedName>
+    <definedName name="TERM_G">Assumptions!$C$87</definedName>
+    <definedName name="KE">Assumptions!$C$82</definedName>
+    <definedName name="KD">Assumptions!$C$83</definedName>
+    <definedName name="RF_RATE">Assumptions!$C$75</definedName>
+    <definedName name="ERP">Assumptions!$C$76</definedName>
+    <definedName name="BETA_U">Assumptions!$C$77</definedName>
+    <definedName name="TAX_RATE_Y1">Assumptions!$C$37</definedName>
+    <definedName name="PAYOUT_Y1">Assumptions!$C$57</definedName>
+    <definedName name="MIN_CASH_PCT">Assumptions!$C$61</definedName>
+    <definedName name="SHARES_DIL">Equity_Roll!$C$21</definedName>
+    <definedName name="DCF_PS">DCF!$D$25</definedName>
+    <definedName name="FCFE_PS">FCFE!$D$18</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" iterate="1" iterateCount="1000" iterateDelta="0.0001"/>
 </workbook>
 </file>
@@ -872,7 +889,7 @@
         </is>
       </c>
       <c r="C24" s="4">
-        <f>TEXT(Summary!C11,"0.00")&amp;" ~ "&amp;TEXT(Summary!D11,"0.00")</f>
+        <f>TEXT(Summary!C12,"0.00")&amp;" ~ "&amp;TEXT(Summary!D12,"0.00")</f>
         <v/>
       </c>
     </row>
@@ -883,7 +900,7 @@
         </is>
       </c>
       <c r="C25" s="4">
-        <f>Checks!F22</f>
+        <f>Checks!F24</f>
         <v/>
       </c>
     </row>
@@ -5866,6 +5883,487 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:J21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="60" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>沪电股份 — FCFE 股权自由现金流估值 (Ke折现, 与FCFF双视图)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="14" customHeight="1">
+      <c r="A2" s="11" t="inlineStr">
+        <is>
+          <t>单位: 人民币百万元 | FCFE=归母净利+D&amp;A-ΔNWC-Capex+净新增借款(FIN页调度); 按股权成本Ke折现(年中口径与DCF页一致), 直接得股权价值, 无需EV→Equity桥</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>项目</t>
+        </is>
+      </c>
+      <c r="E3" s="12" t="inlineStr">
+        <is>
+          <t>2026E</t>
+        </is>
+      </c>
+      <c r="F3" s="12" t="inlineStr">
+        <is>
+          <t>2027E</t>
+        </is>
+      </c>
+      <c r="G3" s="12" t="inlineStr">
+        <is>
+          <t>2028E</t>
+        </is>
+      </c>
+      <c r="H3" s="12" t="inlineStr">
+        <is>
+          <t>2029E</t>
+        </is>
+      </c>
+      <c r="I3" s="12" t="inlineStr">
+        <is>
+          <t>2030E</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>备注</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>归母净利润</t>
+        </is>
+      </c>
+      <c r="E4" s="26">
+        <f>IS!E20</f>
+        <v/>
+      </c>
+      <c r="F4" s="26">
+        <f>IS!F20</f>
+        <v/>
+      </c>
+      <c r="G4" s="26">
+        <f>IS!G20</f>
+        <v/>
+      </c>
+      <c r="H4" s="26">
+        <f>IS!H20</f>
+        <v/>
+      </c>
+      <c r="I4" s="26">
+        <f>IS!I20</f>
+        <v/>
+      </c>
+      <c r="J4" s="11" t="inlineStr">
+        <is>
+          <t>＝IS归母净利(含FIN调度后的利息)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>加: D&amp;A</t>
+        </is>
+      </c>
+      <c r="E5" s="26">
+        <f>PPE!E19</f>
+        <v/>
+      </c>
+      <c r="F5" s="26">
+        <f>PPE!F19</f>
+        <v/>
+      </c>
+      <c r="G5" s="26">
+        <f>PPE!G19</f>
+        <v/>
+      </c>
+      <c r="H5" s="26">
+        <f>PPE!H19</f>
+        <v/>
+      </c>
+      <c r="I5" s="26">
+        <f>PPE!I19</f>
+        <v/>
+      </c>
+      <c r="J5" s="11" t="inlineStr">
+        <is>
+          <t>＝PP&amp;E页折旧+无形摊销</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>减: ΔNWC</t>
+        </is>
+      </c>
+      <c r="E6" s="26">
+        <f>Schedules!E18</f>
+        <v/>
+      </c>
+      <c r="F6" s="26">
+        <f>Schedules!F18</f>
+        <v/>
+      </c>
+      <c r="G6" s="26">
+        <f>Schedules!G18</f>
+        <v/>
+      </c>
+      <c r="H6" s="26">
+        <f>Schedules!H18</f>
+        <v/>
+      </c>
+      <c r="I6" s="26">
+        <f>Schedules!I18</f>
+        <v/>
+      </c>
+      <c r="J6" s="11" t="inlineStr">
+        <is>
+          <t>＝Schedules; NWC增加为现金流出</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>减: Capex</t>
+        </is>
+      </c>
+      <c r="E7" s="26">
+        <f>PPE!E14</f>
+        <v/>
+      </c>
+      <c r="F7" s="26">
+        <f>PPE!F14</f>
+        <v/>
+      </c>
+      <c r="G7" s="26">
+        <f>PPE!G14</f>
+        <v/>
+      </c>
+      <c r="H7" s="26">
+        <f>PPE!H14</f>
+        <v/>
+      </c>
+      <c r="I7" s="26">
+        <f>PPE!I14</f>
+        <v/>
+      </c>
+      <c r="J7" s="11" t="inlineStr">
+        <is>
+          <t>＝PP&amp;E页资本开支</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>加: 净新增借款</t>
+        </is>
+      </c>
+      <c r="E8" s="26">
+        <f>FIN!E57</f>
+        <v/>
+      </c>
+      <c r="F8" s="26">
+        <f>FIN!F57</f>
+        <v/>
+      </c>
+      <c r="G8" s="26">
+        <f>FIN!G57</f>
+        <v/>
+      </c>
+      <c r="H8" s="26">
+        <f>FIN!H57</f>
+        <v/>
+      </c>
+      <c r="I8" s="26">
+        <f>FIN!I57</f>
+        <v/>
+      </c>
+      <c r="J8" s="11" t="inlineStr">
+        <is>
+          <t>＝FIN四档债务期末-期初(revolver新增-sweep偿还-计划还款); 股权口径下债务净变动归股东</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>FCFE</t>
+        </is>
+      </c>
+      <c r="E9" s="35">
+        <f>E4+E5-E6-E7+E8</f>
+        <v/>
+      </c>
+      <c r="F9" s="35">
+        <f>F4+F5-F6-F7+F8</f>
+        <v/>
+      </c>
+      <c r="G9" s="35">
+        <f>G4+G5-G6-G7+G8</f>
+        <v/>
+      </c>
+      <c r="H9" s="35">
+        <f>H4+H5-H6-H7+H8</f>
+        <v/>
+      </c>
+      <c r="I9" s="35">
+        <f>I4+I5-I6-I7+I8</f>
+        <v/>
+      </c>
+      <c r="J9" s="11" t="inlineStr">
+        <is>
+          <t>＝归母+D&amp;A-ΔNWC-Capex+净新增借款</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>折现年序(年中)</t>
+        </is>
+      </c>
+      <c r="E10" s="41" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F10" s="41" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G10" s="41" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="H10" s="41" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="I10" s="41" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="J10" s="11" t="inlineStr">
+        <is>
+          <t>年中折现, 与DCF页同口径</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>折现因子 (Ke)</t>
+        </is>
+      </c>
+      <c r="E11" s="31">
+        <f>1/(1+KE)^E10</f>
+        <v/>
+      </c>
+      <c r="F11" s="31">
+        <f>1/(1+KE)^F10</f>
+        <v/>
+      </c>
+      <c r="G11" s="31">
+        <f>1/(1+KE)^G10</f>
+        <v/>
+      </c>
+      <c r="H11" s="31">
+        <f>1/(1+KE)^H10</f>
+        <v/>
+      </c>
+      <c r="I11" s="31">
+        <f>1/(1+KE)^I10</f>
+        <v/>
+      </c>
+      <c r="J11" s="11" t="inlineStr">
+        <is>
+          <t>＝1/(1+Ke)^t; Ke为named range(Assumptions股权成本)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>PV(FCFE)</t>
+        </is>
+      </c>
+      <c r="E12" s="26">
+        <f>E9*E11</f>
+        <v/>
+      </c>
+      <c r="F12" s="26">
+        <f>F9*F11</f>
+        <v/>
+      </c>
+      <c r="G12" s="26">
+        <f>G9*G11</f>
+        <v/>
+      </c>
+      <c r="H12" s="26">
+        <f>H9*H11</f>
+        <v/>
+      </c>
+      <c r="I12" s="26">
+        <f>I9*I11</f>
+        <v/>
+      </c>
+      <c r="J12" s="11" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>显性期PV合计 (2026-2030)</t>
+        </is>
+      </c>
+      <c r="D14" s="35">
+        <f>SUM(E12:I12)</f>
+        <v/>
+      </c>
+      <c r="J14" s="11" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>终值 TV (Gordon)</t>
+        </is>
+      </c>
+      <c r="D15" s="26">
+        <f>I9*(1+TERM_G)/(KE-TERM_G)</f>
+        <v/>
+      </c>
+      <c r="J15" s="11" t="inlineStr">
+        <is>
+          <t>＝FCFE2030×(1+g)/(Ke-g); Ke/g均为named range</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>PV(终值)</t>
+        </is>
+      </c>
+      <c r="D16" s="26">
+        <f>D15*I11</f>
+        <v/>
+      </c>
+      <c r="J16" s="11" t="inlineStr">
+        <is>
+          <t>终值按t=4.5折现(与DCF页一致)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>股权价值 (FCFE口径)</t>
+        </is>
+      </c>
+      <c r="D17" s="35">
+        <f>D14+D16</f>
+        <v/>
+      </c>
+      <c r="J17" s="11" t="inlineStr">
+        <is>
+          <t>FCFE直接折现为股权价值, 无需净现金桥</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>每股价值 (元)</t>
+        </is>
+      </c>
+      <c r="D18" s="15">
+        <f>D17/SHARES_DIL</f>
+        <v/>
+      </c>
+      <c r="J18" s="11" t="inlineStr">
+        <is>
+          <t>＝股权价值/稀释股数(named range)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>对照: FCFF口径每股价值 (元)</t>
+        </is>
+      </c>
+      <c r="D19" s="14">
+        <f>DCF!D25</f>
+        <v/>
+      </c>
+      <c r="J19" s="11" t="inlineStr">
+        <is>
+          <t>＝DCF页主输出</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>两法差异 (FCFE/FCFF-1)</t>
+        </is>
+      </c>
+      <c r="D20" s="42">
+        <f>D18/D19-1</f>
+        <v/>
+      </c>
+      <c r="J20" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Checks页含一致性信息行</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="52" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>两法差异原因</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>①折现率不同: FCFF按WACC(全资本成本, 税盾在分母)折现, FCFE按Ke(纯股权成本)折现; ②口径不同: FCFF为企业自由现金流, 须经EV→Equity桥加回净现金/扣有息负债, FCFE已含净新增借款、直接对应股权; ③杠杆路径不同: FCFE逐年反映FIN页revolver/sweep实际债务调度(资本结构动态变化), FCFF隐含目标结构(Wd)恒定; ④两法在"恒定资本结构+一致税盾处理"下理论等价, 实务差异主要来自债务调度时点、净现金桥与折现率差; 差异幅度大时应复查融资假设</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="B21:J21"/>
+    <mergeCell ref="A2:J2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:O19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -6393,7 +6891,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6894,7 +7392,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7645,13 +8143,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J23"/>
+  <dimension ref="A1:J25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -8072,132 +8570,168 @@
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>信息项: 隐含折旧率(折旧/期初固资净值)</t>
-        </is>
-      </c>
-      <c r="E16" s="55">
-        <f>PPE!E20</f>
-        <v/>
-      </c>
-      <c r="F16" s="55">
-        <f>PPE!F20</f>
-        <v/>
-      </c>
-      <c r="G16" s="55">
-        <f>PPE!G20</f>
-        <v/>
-      </c>
-      <c r="H16" s="55">
-        <f>PPE!H20</f>
-        <v/>
-      </c>
-      <c r="I16" s="55">
-        <f>PPE!I20</f>
-        <v/>
-      </c>
-      <c r="J16" s="11" t="inlineStr">
-        <is>
-          <t>信息行: 合理带宽8%-18%</t>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>12. Named ranges存在性 (审计轨迹, 15个)</t>
+        </is>
+      </c>
+      <c r="B15" s="54">
+        <f>AND(ISNUMBER(INDIRECT("SCEN_SWITCH")),ISNUMBER(INDIRECT("WACC_USED")),ISNUMBER(INDIRECT("WACC_CALC")),ISNUMBER(INDIRECT("TERM_G")),ISNUMBER(INDIRECT("KE")),ISNUMBER(INDIRECT("KD")),ISNUMBER(INDIRECT("RF_RATE")),ISNUMBER(INDIRECT("ERP")),ISNUMBER(INDIRECT("BETA_U")),ISNUMBER(INDIRECT("TAX_RATE_Y1")),ISNUMBER(INDIRECT("PAYOUT_Y1")),ISNUMBER(INDIRECT("MIN_CASH_PCT")),ISNUMBER(INDIRECT("SHARES_DIL")),ISNUMBER(INDIRECT("DCF_PS")),ISNUMBER(INDIRECT("FCFE_PS")))</f>
+        <v/>
+      </c>
+      <c r="J15" s="11" t="inlineStr">
+        <is>
+          <t>WACC采用值/永续g/Ke/Kd/rf/ERP/βu/税率/股利/最低现金/情景开关/稀释股数/DCF&amp;FCFE每股; 任一named range被删则FALSE</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>信息项: 2026E模型收入/一致预期</t>
-        </is>
-      </c>
-      <c r="B17" s="16">
-        <f>IS!E4/Assumptions!$C$12</f>
+          <t>信息项: 隐含折旧率(折旧/期初固资净值)</t>
+        </is>
+      </c>
+      <c r="E17" s="55">
+        <f>PPE!E20</f>
+        <v/>
+      </c>
+      <c r="F17" s="55">
+        <f>PPE!F20</f>
+        <v/>
+      </c>
+      <c r="G17" s="55">
+        <f>PPE!G20</f>
+        <v/>
+      </c>
+      <c r="H17" s="55">
+        <f>PPE!H20</f>
+        <v/>
+      </c>
+      <c r="I17" s="55">
+        <f>PPE!I20</f>
         <v/>
       </c>
       <c r="J17" s="11" t="inlineStr">
         <is>
-          <t>接近100%即基准贴合一致预期</t>
+          <t>信息行: 合理带宽8%-18%</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>信息项: 2026E模型归母/一致预期</t>
+          <t>信息项: 2026E模型收入/一致预期</t>
         </is>
       </c>
       <c r="B18" s="16">
-        <f>IS!E20/Assumptions!$C$13</f>
-        <v/>
+        <f>IS!E4/Assumptions!$C$12</f>
+        <v/>
+      </c>
+      <c r="J18" s="11" t="inlineStr">
+        <is>
+          <t>接近100%即基准贴合一致预期</t>
+        </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>信息项: WACC计算值/采用值</t>
+          <t>信息项: 2026E模型归母/一致预期</t>
         </is>
       </c>
       <c r="B19" s="16">
-        <f>Assumptions!C84</f>
-        <v/>
-      </c>
-      <c r="C19" s="16">
-        <f>Assumptions!C86</f>
-        <v/>
-      </c>
-      <c r="J19" s="11" t="inlineStr">
-        <is>
-          <t>左=计算值, 右=采用值(override为空时两者相等)</t>
-        </is>
+        <f>IS!E20/Assumptions!$C$13</f>
+        <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
+          <t>信息项: WACC计算值/采用值</t>
+        </is>
+      </c>
+      <c r="B20" s="16">
+        <f>Assumptions!C84</f>
+        <v/>
+      </c>
+      <c r="C20" s="16">
+        <f>Assumptions!C86</f>
+        <v/>
+      </c>
+      <c r="J20" s="11" t="inlineStr">
+        <is>
+          <t>左=计算值, 右=采用值(override为空时两者相等)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>信息项: FCFE/FCFF每股价值比</t>
+        </is>
+      </c>
+      <c r="B21" s="16">
+        <f>FCFE!D18/DCF!D25</f>
+        <v/>
+      </c>
+      <c r="C21" s="14">
+        <f>FCFE!D18</f>
+        <v/>
+      </c>
+      <c r="J21" s="11" t="inlineStr">
+        <is>
+          <t>左=FCFE/FCFF比值, 右=FCFE每股(元); 两法差异原因见FCFE页底部注记</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
           <t>信息项: 2030E现金 vs 最低现金</t>
         </is>
       </c>
-      <c r="B20" s="26">
+      <c r="B22" s="26">
         <f>BS!I4</f>
         <v/>
       </c>
-      <c r="C20" s="26">
+      <c r="C22" s="26">
         <f>FIN!I13</f>
         <v/>
       </c>
-      <c r="J20" s="11" t="inlineStr">
+      <c r="J22" s="11" t="inlineStr">
         <is>
           <t>两者应相等(sweep后现金=最低现金, 溢出去理财)</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="30" customHeight="1">
-      <c r="A22" s="56" t="inlineStr">
+    <row r="24" ht="30" customHeight="1">
+      <c r="A24" s="56" t="inlineStr">
         <is>
           <t xml:space="preserve">汇总: 全部通过 = </t>
         </is>
       </c>
-      <c r="F22" s="57">
-        <f>IF(AND(B4:I4,E5:I5,E6:I6,B7:I7,B8:I8,B9,B10,B11,E12:I12,E13:I13,E14:I14),"全部通过=TRUE","存在未通过=FALSE")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr">
+      <c r="F24" s="57">
+        <f>IF(AND(B4:I4,E5:I5,E6:I6,B7:I7,B8:I8,B9,B10,B11,E12:I12,E13:I13,E14:I14,B15),"全部通过=TRUE","存在未通过=FALSE")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
         <is>
           <t>布尔汇总</t>
         </is>
       </c>
-      <c r="F23" s="27">
-        <f>AND(B4:I4,E5:I5,E6:I6,B7:I7,B8:I8,B9,B10,B11,E12:I12,E13:I13,E14:I14)</f>
+      <c r="F25" s="27">
+        <f>AND(B4:I4,E5:I5,E6:I6,B7:I7,B8:I8,B9,B10,B11,E12:I12,E13:I13,E14:I14,B15)</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A22:E22"/>
-    <mergeCell ref="F22:H22"/>
+    <mergeCell ref="A24:E24"/>
+    <mergeCell ref="F24:H24"/>
     <mergeCell ref="A2:J2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -8210,7 +8744,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -8441,147 +8975,192 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>现价 (2026-08-17)</t>
+          <t>FCFE股权现金流 — 基准</t>
+        </is>
+      </c>
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>Ke折现(股权口径)</t>
         </is>
       </c>
       <c r="C10" s="14">
-        <f>Assumptions!$C$7</f>
+        <f>FCFE!D18</f>
         <v/>
       </c>
       <c r="D10" s="14">
-        <f>Assumptions!$C$7</f>
-        <v/>
-      </c>
-      <c r="E10" s="14">
-        <f>Assumptions!$C$7</f>
-        <v/>
+        <f>FCFE!D18</f>
+        <v/>
+      </c>
+      <c r="E10" s="15">
+        <f>(C10+D10)/2</f>
+        <v/>
+      </c>
+      <c r="F10" s="16">
+        <f>E10/Assumptions!$C$7-1</f>
+        <v/>
+      </c>
+      <c r="G10" s="9" t="inlineStr">
+        <is>
+          <t>FCFE=归母+D&amp;A-ΔNWC-Capex+净新增借款(FIN调度), 与FCFF双视图对照</t>
+        </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
+          <t>现价 (2026-08-17)</t>
+        </is>
+      </c>
+      <c r="C11" s="14">
+        <f>Assumptions!$C$7</f>
+        <v/>
+      </c>
+      <c r="D11" s="14">
+        <f>Assumptions!$C$7</f>
+        <v/>
+      </c>
+      <c r="E11" s="14">
+        <f>Assumptions!$C$7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
           <t>综合参考区间(全方法包络)</t>
         </is>
       </c>
-      <c r="C11" s="17">
-        <f>MIN(C5:C9)</f>
-        <v/>
-      </c>
-      <c r="D11" s="17">
-        <f>MAX(D5:D9)</f>
-        <v/>
-      </c>
-      <c r="E11" s="17">
-        <f>(C11+D11)/2</f>
-        <v/>
-      </c>
-      <c r="F11" s="18">
-        <f>E11/Assumptions!$C$7-1</f>
-        <v/>
-      </c>
-      <c r="G11" s="11" t="inlineStr">
+      <c r="C12" s="17">
+        <f>MIN(C5:C10)</f>
+        <v/>
+      </c>
+      <c r="D12" s="17">
+        <f>MAX(D5:D10)</f>
+        <v/>
+      </c>
+      <c r="E12" s="17">
+        <f>(C12+D12)/2</f>
+        <v/>
+      </c>
+      <c r="F12" s="18">
+        <f>E12/Assumptions!$C$7-1</f>
+        <v/>
+      </c>
+      <c r="G12" s="11" t="inlineStr">
         <is>
           <t>熊简化法DCF下限 ~ 牛简化法/相对估值上限的包络</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="16" customHeight="1">
-      <c r="A13" s="19" t="inlineStr">
+    <row r="14" ht="16" customHeight="1">
+      <c r="A14" s="19" t="inlineStr">
         <is>
           <t>区间可视化 (每个▮≈10元, 起点=区间低值)</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>方法</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>区间条(低→高, 括号为现价相对位置)</t>
         </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="11" t="inlineStr">
-        <is>
-          <t>DCF绝对估值 — 基准</t>
-        </is>
-      </c>
-      <c r="B15" s="20">
-        <f>REPT("▮",MAX(1,ROUND((D5-C5)/10,0)))&amp;"  ["&amp;TEXT(C5,"0")&amp;"—"&amp;TEXT(D5,"0")&amp;"]"</f>
-        <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="11" t="inlineStr">
         <is>
-          <t>DCF绝对估值 — 熊市</t>
+          <t>DCF绝对估值 — 基准</t>
         </is>
       </c>
       <c r="B16" s="20">
-        <f>REPT("▮",MAX(1,ROUND((D6-C6)/10,0)))&amp;"  ["&amp;TEXT(C6,"0")&amp;"—"&amp;TEXT(D6,"0")&amp;"]"</f>
+        <f>REPT("▮",MAX(1,ROUND((D5-C5)/10,0)))&amp;"  ["&amp;TEXT(C5,"0")&amp;"—"&amp;TEXT(D5,"0")&amp;"]"</f>
         <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="11" t="inlineStr">
         <is>
-          <t>DCF绝对估值 — 牛市</t>
+          <t>DCF绝对估值 — 熊市</t>
         </is>
       </c>
       <c r="B17" s="20">
-        <f>REPT("▮",MAX(1,ROUND((D7-C7)/10,0)))&amp;"  ["&amp;TEXT(C7,"0")&amp;"—"&amp;TEXT(D7,"0")&amp;"]"</f>
+        <f>REPT("▮",MAX(1,ROUND((D6-C6)/10,0)))&amp;"  ["&amp;TEXT(C6,"0")&amp;"—"&amp;TEXT(D6,"0")&amp;"]"</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="11" t="inlineStr">
         <is>
-          <t>相对估值 — 模型2026E归母</t>
+          <t>DCF绝对估值 — 牛市</t>
         </is>
       </c>
       <c r="B18" s="20">
-        <f>REPT("▮",MAX(1,ROUND((D8-C8)/10,0)))&amp;"  ["&amp;TEXT(C8,"0")&amp;"—"&amp;TEXT(D8,"0")&amp;"]"</f>
+        <f>REPT("▮",MAX(1,ROUND((D7-C7)/10,0)))&amp;"  ["&amp;TEXT(C7,"0")&amp;"—"&amp;TEXT(D7,"0")&amp;"]"</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="11" t="inlineStr">
         <is>
+          <t>相对估值 — 模型2026E归母</t>
+        </is>
+      </c>
+      <c r="B19" s="20">
+        <f>REPT("▮",MAX(1,ROUND((D8-C8)/10,0)))&amp;"  ["&amp;TEXT(C8,"0")&amp;"—"&amp;TEXT(D8,"0")&amp;"]"</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="11" t="inlineStr">
+        <is>
           <t>相对估值 — 一致预期2026E归母</t>
         </is>
       </c>
-      <c r="B19" s="20">
+      <c r="B20" s="20">
         <f>REPT("▮",MAX(1,ROUND((D9-C9)/10,0)))&amp;"  ["&amp;TEXT(C9,"0")&amp;"—"&amp;TEXT(D9,"0")&amp;"]"</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="inlineStr">
+      <c r="A21" s="11" t="inlineStr">
+        <is>
+          <t>FCFE股权现金流 — 基准</t>
+        </is>
+      </c>
+      <c r="B21" s="20">
+        <f>REPT("▮",MAX(1,ROUND((D10-C10)/10,0)))&amp;"  ["&amp;TEXT(C10,"0")&amp;"—"&amp;TEXT(D10,"0")&amp;"]"</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>关键假设提示</t>
         </is>
       </c>
-      <c r="B21" s="9" t="inlineStr">
+      <c r="B23" s="9" t="inlineStr">
         <is>
           <t>WACC采用值与可比beta联动(Assumptions第十节); 三情景主模型切换见Assumptions情景开关; 校验状态见Checks页</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="10">
     <mergeCell ref="B16:G16"/>
     <mergeCell ref="B19:G19"/>
+    <mergeCell ref="B20:G20"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="B17:G17"/>
-    <mergeCell ref="A13:H13"/>
+    <mergeCell ref="B23:G23"/>
+    <mergeCell ref="A14:H14"/>
     <mergeCell ref="B18:G18"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="B21:G21"/>
-    <mergeCell ref="B15:G15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs(release): 0.3.1 — 00981重生成重验 + examples刷新 + 文档同步
- configs/00981.yaml: 分页修复后重新生成(2023年三表补全, CF 6215.1百万美元
  与BS勾稽), 回贴分析师修正(偿债滚动续作+最低现金60%)
- examples/: 三成稿xlsx/addr/verify日志刷新至0.3.1, LO重算全ALL PASS;
  00981 DCF 1.6233美元/FCFE 0.6769; 002463 DCF 112.2842(mi入桥-0.008);
  300476 DCF精确340.415208186145, 与0.3.0成稿除新增行外数值零差异
- README: 验证记录/方法论/数据口径/Web无鉴权声明同步; AGENTS: pytest与分层依赖;
  CHANGELOG: 0.3.1条目
</commit_message>
<xml_diff>
--- a/examples/002463_沪电股份_估值模型.xlsx
+++ b/examples/002463_沪电股份_估值模型.xlsx
@@ -1,29 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revenue_Segments" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IS" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BS" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CF" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Schedules" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PPE" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FIN" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equity_Roll" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FCFE" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relative_Val" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenarios" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="Cover" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Assumptions" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Revenue_Segments" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="IS" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="BS" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="CF" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Schedules" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="PPE" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="FIN" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Equity_Roll" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="DCF" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="FCFE" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Relative_Val" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Sensitivity" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Scenarios" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="Checks" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames>
     <definedName name="SCEN_SWITCH">Assumptions!$C$5</definedName>
@@ -39,8 +39,8 @@
     <definedName name="PAYOUT_Y1">Assumptions!$C$57</definedName>
     <definedName name="MIN_CASH_PCT">Assumptions!$C$61</definedName>
     <definedName name="SHARES_DIL">Equity_Roll!$C$21</definedName>
-    <definedName name="DCF_PS">DCF!$D$25</definedName>
-    <definedName name="FCFE_PS">FCFE!$D$18</definedName>
+    <definedName name="DCF_PS">DCF!$D$26</definedName>
+    <definedName name="FCFE_PS">FCFE!$D$20</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" iterate="1" iterateCount="1000" iterateDelta="0.0001"/>
 </workbook>
@@ -856,7 +856,7 @@
         </is>
       </c>
       <c r="C21" s="4">
-        <f>DCF!D25</f>
+        <f>DCF!D26</f>
         <v/>
       </c>
     </row>
@@ -942,7 +942,7 @@
     <row r="32" ht="40" customHeight="1">
       <c r="B32" s="7" t="inlineStr">
         <is>
-          <t>5. DCF年中折现: 估值基准日2026-08-17, t=0.5/1.5/.../4.5; EV→Equity桥含货币资金/交易性金融资产/其他权益工具投资/有息负债;</t>
+          <t>5. DCF年中折现: 估值基准日2026-08-17, t=0.5/1.5/.../4.5; EV→Equity桥含货币资金/交易性金融资产/其他权益工具投资/有息负债/少数股东权益;</t>
         </is>
       </c>
     </row>
@@ -5303,7 +5303,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J30"/>
+  <dimension ref="A1:J31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5767,101 +5767,117 @@
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
+          <t>减: 少数股东权益(2025A末)</t>
+        </is>
+      </c>
+      <c r="D23" s="26">
+        <f>-BS!D44</f>
+        <v/>
+      </c>
+      <c r="J23" s="11" t="inlineStr">
+        <is>
+          <t>EV桥得归母口径股权价值须扣少数股东权益(账面值); 无少数股东权益的标的为0, 不影响结果</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
           <t>净现金调整合计</t>
         </is>
       </c>
-      <c r="D23" s="26">
-        <f>D19+D20+D21+D22</f>
-        <v/>
-      </c>
-      <c r="J23" s="11" t="inlineStr">
+      <c r="D24" s="26">
+        <f>D19+D20+D21+D22+D23</f>
+        <v/>
+      </c>
+      <c r="J24" s="11" t="inlineStr">
         <is>
           <t>供Sensitivity/Scenarios页引用</t>
         </is>
       </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="3" t="inlineStr">
-        <is>
-          <t>股权价值</t>
-        </is>
-      </c>
-      <c r="D24" s="35">
-        <f>D18+D23</f>
-        <v/>
-      </c>
-      <c r="J24" s="11" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
+          <t>股权价值</t>
+        </is>
+      </c>
+      <c r="D25" s="35">
+        <f>D18+D24</f>
+        <v/>
+      </c>
+      <c r="J25" s="11" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
           <t>每股价值 (元)</t>
         </is>
       </c>
-      <c r="D25" s="15">
-        <f>D24/Equity_Roll!$C$21</f>
-        <v/>
-      </c>
-      <c r="J25" s="11" t="inlineStr">
+      <c r="D26" s="15">
+        <f>D25/Equity_Roll!$C$21</f>
+        <v/>
+      </c>
+      <c r="J26" s="11" t="inlineStr">
         <is>
           <t>＝股权价值/稀释股数(Equity_Roll页)</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="4" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
         <is>
           <t>现价 (2026-08-17)</t>
         </is>
       </c>
-      <c r="D26" s="14">
+      <c r="D27" s="14">
         <f>Assumptions!$C$7</f>
         <v/>
       </c>
-      <c r="J26" s="11" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="3" t="inlineStr">
+      <c r="J27" s="11" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
         <is>
           <t>隐含涨跌幅</t>
         </is>
       </c>
-      <c r="D27" s="42">
-        <f>D25/D26-1</f>
-        <v/>
-      </c>
-      <c r="J27" s="11" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="4" t="inlineStr">
-        <is>
-          <t>隐含2026E P/E</t>
-        </is>
-      </c>
-      <c r="D28" s="43">
-        <f>D24/IS!E20</f>
-        <v/>
-      </c>
-      <c r="J28" s="11" t="inlineStr">
-        <is>
-          <t>＝股权价值/2026E归母</t>
-        </is>
-      </c>
+      <c r="D28" s="42">
+        <f>D26/D27-1</f>
+        <v/>
+      </c>
+      <c r="J28" s="11" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
+          <t>隐含2026E P/E</t>
+        </is>
+      </c>
+      <c r="D29" s="43">
+        <f>D25/IS!E20</f>
+        <v/>
+      </c>
+      <c r="J29" s="11" t="inlineStr">
+        <is>
+          <t>＝股权价值/2026E归母</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
           <t>隐含2026E EV/EBITDA</t>
         </is>
       </c>
-      <c r="D29" s="43">
+      <c r="D30" s="43">
         <f>D18/(IS!E23+PPE!E19)</f>
         <v/>
       </c>
-      <c r="J29" s="11" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="11" t="inlineStr">
+      <c r="J30" s="11" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="11" t="inlineStr">
         <is>
           <t>注: 估值基准日2026-08-17, 与2026财年现金流起点存在时间错位; 年中折现(t=0.5起)为该错位的标准近似处理, 不再单独做stub调整</t>
         </is>
@@ -5870,7 +5886,7 @@
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A30:J30"/>
+    <mergeCell ref="A31:J31"/>
     <mergeCell ref="A2:J2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5883,7 +5899,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J21"/>
+  <dimension ref="A1:J23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5908,7 +5924,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="11" t="inlineStr">
         <is>
-          <t>单位: 人民币百万元 | FCFE=归母净利+D&amp;A-ΔNWC-Capex+净新增借款(FIN页调度); 按股权成本Ke折现(年中口径与DCF页一致), 直接得股权价值, 无需EV→Equity桥</t>
+          <t>单位: 人民币百万元 | FCFE=归母净利+D&amp;A-ΔNWC-Capex+净新增借款(FIN页调度); 按股权成本Ke折现(年中口径与DCF页一致), 直接得归母股权价值(少数股东权益见DCF页EV→Equity桥); 终值取正常化FCFE(净新增借款按g封顶)</t>
         </is>
       </c>
     </row>
@@ -6110,248 +6126,296 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>理财净变动(勾稽参考, 不计入FCFE)</t>
+        </is>
+      </c>
+      <c r="E9" s="26">
+        <f>-FIN!E62</f>
+        <v/>
+      </c>
+      <c r="F9" s="26">
+        <f>-FIN!F62</f>
+        <v/>
+      </c>
+      <c r="G9" s="26">
+        <f>-FIN!G62</f>
+        <v/>
+      </c>
+      <c r="H9" s="26">
+        <f>-FIN!H62</f>
+        <v/>
+      </c>
+      <c r="I9" s="26">
+        <f>-FIN!I62</f>
+        <v/>
+      </c>
+      <c r="J9" s="11" t="inlineStr">
+        <is>
+          <t>＝-FIN理财净变动: sweep溢出购买理财为现金↔理财的形态转换(资产仍在表内归属股东), 故不计入FCFE; 显性列示供FCFE↔FCFF差异勾稽(FCFF也未扣理财购买, 两法在此口径一致)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>FCFE</t>
         </is>
       </c>
-      <c r="E9" s="35">
+      <c r="E10" s="35">
         <f>E4+E5-E6-E7+E8</f>
         <v/>
       </c>
-      <c r="F9" s="35">
+      <c r="F10" s="35">
         <f>F4+F5-F6-F7+F8</f>
         <v/>
       </c>
-      <c r="G9" s="35">
+      <c r="G10" s="35">
         <f>G4+G5-G6-G7+G8</f>
         <v/>
       </c>
-      <c r="H9" s="35">
+      <c r="H10" s="35">
         <f>H4+H5-H6-H7+H8</f>
         <v/>
       </c>
-      <c r="I9" s="35">
+      <c r="I10" s="35">
         <f>I4+I5-I6-I7+I8</f>
         <v/>
       </c>
-      <c r="J9" s="11" t="inlineStr">
+      <c r="J10" s="11" t="inlineStr">
         <is>
           <t>＝归母+D&amp;A-ΔNWC-Capex+净新增借款</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>折现年序(年中)</t>
-        </is>
-      </c>
-      <c r="E10" s="41" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="F10" s="41" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="G10" s="41" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="H10" s="41" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="I10" s="41" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="J10" s="11" t="inlineStr">
-        <is>
-          <t>年中折现, 与DCF页同口径</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>折现因子 (Ke)</t>
-        </is>
-      </c>
-      <c r="E11" s="31">
-        <f>1/(1+KE)^E10</f>
-        <v/>
-      </c>
-      <c r="F11" s="31">
-        <f>1/(1+KE)^F10</f>
-        <v/>
-      </c>
-      <c r="G11" s="31">
-        <f>1/(1+KE)^G10</f>
-        <v/>
-      </c>
-      <c r="H11" s="31">
-        <f>1/(1+KE)^H10</f>
-        <v/>
-      </c>
-      <c r="I11" s="31">
-        <f>1/(1+KE)^I10</f>
-        <v/>
+          <t>折现年序(年中)</t>
+        </is>
+      </c>
+      <c r="E11" s="41" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F11" s="41" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G11" s="41" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="H11" s="41" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="I11" s="41" t="n">
+        <v>4.5</v>
       </c>
       <c r="J11" s="11" t="inlineStr">
         <is>
-          <t>＝1/(1+Ke)^t; Ke为named range(Assumptions股权成本)</t>
+          <t>年中折现, 与DCF页同口径</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
+          <t>折现因子 (Ke)</t>
+        </is>
+      </c>
+      <c r="E12" s="31">
+        <f>1/(1+KE)^E11</f>
+        <v/>
+      </c>
+      <c r="F12" s="31">
+        <f>1/(1+KE)^F11</f>
+        <v/>
+      </c>
+      <c r="G12" s="31">
+        <f>1/(1+KE)^G11</f>
+        <v/>
+      </c>
+      <c r="H12" s="31">
+        <f>1/(1+KE)^H11</f>
+        <v/>
+      </c>
+      <c r="I12" s="31">
+        <f>1/(1+KE)^I11</f>
+        <v/>
+      </c>
+      <c r="J12" s="11" t="inlineStr">
+        <is>
+          <t>＝1/(1+Ke)^t; Ke为named range(Assumptions股权成本)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
           <t>PV(FCFE)</t>
         </is>
       </c>
-      <c r="E12" s="26">
-        <f>E9*E11</f>
-        <v/>
-      </c>
-      <c r="F12" s="26">
-        <f>F9*F11</f>
-        <v/>
-      </c>
-      <c r="G12" s="26">
-        <f>G9*G11</f>
-        <v/>
-      </c>
-      <c r="H12" s="26">
-        <f>H9*H11</f>
-        <v/>
-      </c>
-      <c r="I12" s="26">
-        <f>I9*I11</f>
-        <v/>
-      </c>
-      <c r="J12" s="11" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+      <c r="E13" s="26">
+        <f>E10*E12</f>
+        <v/>
+      </c>
+      <c r="F13" s="26">
+        <f>F10*F12</f>
+        <v/>
+      </c>
+      <c r="G13" s="26">
+        <f>G10*G12</f>
+        <v/>
+      </c>
+      <c r="H13" s="26">
+        <f>H10*H12</f>
+        <v/>
+      </c>
+      <c r="I13" s="26">
+        <f>I10*I12</f>
+        <v/>
+      </c>
+      <c r="J13" s="11" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>显性期PV合计 (2026-2030)</t>
         </is>
       </c>
-      <c r="D14" s="35">
-        <f>SUM(E12:I12)</f>
-        <v/>
-      </c>
-      <c r="J14" s="11" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>终值 TV (Gordon)</t>
-        </is>
-      </c>
-      <c r="D15" s="26">
-        <f>I9*(1+TERM_G)/(KE-TERM_G)</f>
-        <v/>
-      </c>
-      <c r="J15" s="11" t="inlineStr">
-        <is>
-          <t>＝FCFE2030×(1+g)/(Ke-g); Ke/g均为named range</t>
-        </is>
-      </c>
+      <c r="D15" s="35">
+        <f>SUM(E13:I13)</f>
+        <v/>
+      </c>
+      <c r="J15" s="11" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
+          <t>正常化FCFE (2030E, 终值口径)</t>
+        </is>
+      </c>
+      <c r="D16" s="26">
+        <f>I10-I8+MIN(I8,FIN!I56*TERM_G)</f>
+        <v/>
+      </c>
+      <c r="J16" s="11" t="inlineStr">
+        <is>
+          <t>净新增借款按g封顶: 终值内净新增借款取MIN(实际调度, 2030E期末有息负债×g), 防止显性期末大额净融资被Gordon公式永续外推; 去杠杆/平稳年(实际≤封顶值)维持实际调度不变</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>终值 TV (Gordon, 正常化FCFE)</t>
+        </is>
+      </c>
+      <c r="D17" s="26">
+        <f>D16*(1+TERM_G)/(KE-TERM_G)</f>
+        <v/>
+      </c>
+      <c r="J17" s="11" t="inlineStr">
+        <is>
+          <t>＝正常化FCFE2030×(1+g)/(Ke-g); Ke/g均为named range</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
           <t>PV(终值)</t>
         </is>
       </c>
-      <c r="D16" s="26">
-        <f>D15*I11</f>
-        <v/>
-      </c>
-      <c r="J16" s="11" t="inlineStr">
+      <c r="D18" s="26">
+        <f>D17*I12</f>
+        <v/>
+      </c>
+      <c r="J18" s="11" t="inlineStr">
         <is>
           <t>终值按t=4.5折现(与DCF页一致)</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>股权价值 (FCFE口径)</t>
         </is>
       </c>
-      <c r="D17" s="35">
-        <f>D14+D16</f>
-        <v/>
-      </c>
-      <c r="J17" s="11" t="inlineStr">
+      <c r="D19" s="35">
+        <f>D15+D18</f>
+        <v/>
+      </c>
+      <c r="J19" s="11" t="inlineStr">
         <is>
           <t>FCFE直接折现为股权价值, 无需净现金桥</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>每股价值 (元)</t>
-        </is>
-      </c>
-      <c r="D18" s="15">
-        <f>D17/SHARES_DIL</f>
-        <v/>
-      </c>
-      <c r="J18" s="11" t="inlineStr">
-        <is>
-          <t>＝股权价值/稀释股数(named range)</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>对照: FCFF口径每股价值 (元)</t>
-        </is>
-      </c>
-      <c r="D19" s="14">
-        <f>DCF!D25</f>
-        <v/>
-      </c>
-      <c r="J19" s="11" t="inlineStr">
-        <is>
-          <t>＝DCF页主输出</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
+          <t>每股价值 (元)</t>
+        </is>
+      </c>
+      <c r="D20" s="15">
+        <f>D19/SHARES_DIL</f>
+        <v/>
+      </c>
+      <c r="J20" s="11" t="inlineStr">
+        <is>
+          <t>＝股权价值/稀释股数(named range)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>对照: FCFF口径每股价值 (元)</t>
+        </is>
+      </c>
+      <c r="D21" s="14">
+        <f>DCF!D26</f>
+        <v/>
+      </c>
+      <c r="J21" s="11" t="inlineStr">
+        <is>
+          <t>＝DCF页主输出</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
           <t>两法差异 (FCFE/FCFF-1)</t>
         </is>
       </c>
-      <c r="D20" s="42">
-        <f>D18/D19-1</f>
-        <v/>
-      </c>
-      <c r="J20" s="11" t="inlineStr">
+      <c r="D22" s="42">
+        <f>D20/D21-1</f>
+        <v/>
+      </c>
+      <c r="J22" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve"> Checks页含一致性信息行</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="52" customHeight="1">
-      <c r="A21" s="3" t="inlineStr">
+    <row r="23" ht="52" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>两法差异原因</t>
         </is>
       </c>
-      <c r="B21" s="9" t="inlineStr">
-        <is>
-          <t>①折现率不同: FCFF按WACC(全资本成本, 税盾在分母)折现, FCFE按Ke(纯股权成本)折现; ②口径不同: FCFF为企业自由现金流, 须经EV→Equity桥加回净现金/扣有息负债, FCFE已含净新增借款、直接对应股权; ③杠杆路径不同: FCFE逐年反映FIN页revolver/sweep实际债务调度(资本结构动态变化), FCFF隐含目标结构(Wd)恒定; ④两法在"恒定资本结构+一致税盾处理"下理论等价, 实务差异主要来自债务调度时点、净现金桥与折现率差; 差异幅度大时应复查融资假设</t>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>①折现率不同: FCFF按WACC(全资本成本, 税盾在分母)折现, FCFE按Ke(纯股权成本)折现; ②口径不同: FCFF为企业自由现金流, 须经EV→Equity桥加回净现金/扣有息负债/扣少数股东权益, FCFE基于归母净利折现、直接对应归母股权价值, 少数股东权益已在DCF页EV→Equity桥扣除, 本页无需再扣; ③杠杆路径不同: FCFE逐年反映FIN页revolver/sweep实际债务调度(资本结构动态变化), FCFF隐含目标结构(Wd)恒定; ④理财净变动(上行勾稽参考行)为现金形态转换, 两法均未计入, 不构成差异来源; ⑤两法在"恒定资本结构+一致税盾处理"下理论等价, 实务差异主要来自债务调度时点、净现金桥与折现率差; 差异幅度大时应复查融资假设</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
+    <mergeCell ref="B23:J23"/>
     <mergeCell ref="A1:J1"/>
-    <mergeCell ref="B21:J21"/>
     <mergeCell ref="A2:J2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6964,23 +7028,23 @@
         <v/>
       </c>
       <c r="C6" s="14">
-        <f>(DCF!$E$10/(1+$B6)^0.5+DCF!$F$10/(1+$B6)^1.5+DCF!$G$10/(1+$B6)^2.5+DCF!$H$10/(1+$B6)^3.5+DCF!$I$10/(1+$B6)^4.5+DCF!$I$10*(1+C$5)/($B6-C$5)/(1+$B6)^4.5+DCF!$D$23)/Equity_Roll!$C$21</f>
+        <f>(DCF!$E$10/(1+$B6)^0.5+DCF!$F$10/(1+$B6)^1.5+DCF!$G$10/(1+$B6)^2.5+DCF!$H$10/(1+$B6)^3.5+DCF!$I$10/(1+$B6)^4.5+DCF!$I$10*(1+C$5)/($B6-C$5)/(1+$B6)^4.5+DCF!$D$24)/Equity_Roll!$C$21</f>
         <v/>
       </c>
       <c r="D6" s="14">
-        <f>(DCF!$E$10/(1+$B6)^0.5+DCF!$F$10/(1+$B6)^1.5+DCF!$G$10/(1+$B6)^2.5+DCF!$H$10/(1+$B6)^3.5+DCF!$I$10/(1+$B6)^4.5+DCF!$I$10*(1+D$5)/($B6-D$5)/(1+$B6)^4.5+DCF!$D$23)/Equity_Roll!$C$21</f>
+        <f>(DCF!$E$10/(1+$B6)^0.5+DCF!$F$10/(1+$B6)^1.5+DCF!$G$10/(1+$B6)^2.5+DCF!$H$10/(1+$B6)^3.5+DCF!$I$10/(1+$B6)^4.5+DCF!$I$10*(1+D$5)/($B6-D$5)/(1+$B6)^4.5+DCF!$D$24)/Equity_Roll!$C$21</f>
         <v/>
       </c>
       <c r="E6" s="14">
-        <f>(DCF!$E$10/(1+$B6)^0.5+DCF!$F$10/(1+$B6)^1.5+DCF!$G$10/(1+$B6)^2.5+DCF!$H$10/(1+$B6)^3.5+DCF!$I$10/(1+$B6)^4.5+DCF!$I$10*(1+E$5)/($B6-E$5)/(1+$B6)^4.5+DCF!$D$23)/Equity_Roll!$C$21</f>
+        <f>(DCF!$E$10/(1+$B6)^0.5+DCF!$F$10/(1+$B6)^1.5+DCF!$G$10/(1+$B6)^2.5+DCF!$H$10/(1+$B6)^3.5+DCF!$I$10/(1+$B6)^4.5+DCF!$I$10*(1+E$5)/($B6-E$5)/(1+$B6)^4.5+DCF!$D$24)/Equity_Roll!$C$21</f>
         <v/>
       </c>
       <c r="F6" s="14">
-        <f>(DCF!$E$10/(1+$B6)^0.5+DCF!$F$10/(1+$B6)^1.5+DCF!$G$10/(1+$B6)^2.5+DCF!$H$10/(1+$B6)^3.5+DCF!$I$10/(1+$B6)^4.5+DCF!$I$10*(1+F$5)/($B6-F$5)/(1+$B6)^4.5+DCF!$D$23)/Equity_Roll!$C$21</f>
+        <f>(DCF!$E$10/(1+$B6)^0.5+DCF!$F$10/(1+$B6)^1.5+DCF!$G$10/(1+$B6)^2.5+DCF!$H$10/(1+$B6)^3.5+DCF!$I$10/(1+$B6)^4.5+DCF!$I$10*(1+F$5)/($B6-F$5)/(1+$B6)^4.5+DCF!$D$24)/Equity_Roll!$C$21</f>
         <v/>
       </c>
       <c r="G6" s="14">
-        <f>(DCF!$E$10/(1+$B6)^0.5+DCF!$F$10/(1+$B6)^1.5+DCF!$G$10/(1+$B6)^2.5+DCF!$H$10/(1+$B6)^3.5+DCF!$I$10/(1+$B6)^4.5+DCF!$I$10*(1+G$5)/($B6-G$5)/(1+$B6)^4.5+DCF!$D$23)/Equity_Roll!$C$21</f>
+        <f>(DCF!$E$10/(1+$B6)^0.5+DCF!$F$10/(1+$B6)^1.5+DCF!$G$10/(1+$B6)^2.5+DCF!$H$10/(1+$B6)^3.5+DCF!$I$10/(1+$B6)^4.5+DCF!$I$10*(1+G$5)/($B6-G$5)/(1+$B6)^4.5+DCF!$D$24)/Equity_Roll!$C$21</f>
         <v/>
       </c>
     </row>
@@ -6990,23 +7054,23 @@
         <v/>
       </c>
       <c r="C7" s="14">
-        <f>(DCF!$E$10/(1+$B7)^0.5+DCF!$F$10/(1+$B7)^1.5+DCF!$G$10/(1+$B7)^2.5+DCF!$H$10/(1+$B7)^3.5+DCF!$I$10/(1+$B7)^4.5+DCF!$I$10*(1+C$5)/($B7-C$5)/(1+$B7)^4.5+DCF!$D$23)/Equity_Roll!$C$21</f>
+        <f>(DCF!$E$10/(1+$B7)^0.5+DCF!$F$10/(1+$B7)^1.5+DCF!$G$10/(1+$B7)^2.5+DCF!$H$10/(1+$B7)^3.5+DCF!$I$10/(1+$B7)^4.5+DCF!$I$10*(1+C$5)/($B7-C$5)/(1+$B7)^4.5+DCF!$D$24)/Equity_Roll!$C$21</f>
         <v/>
       </c>
       <c r="D7" s="14">
-        <f>(DCF!$E$10/(1+$B7)^0.5+DCF!$F$10/(1+$B7)^1.5+DCF!$G$10/(1+$B7)^2.5+DCF!$H$10/(1+$B7)^3.5+DCF!$I$10/(1+$B7)^4.5+DCF!$I$10*(1+D$5)/($B7-D$5)/(1+$B7)^4.5+DCF!$D$23)/Equity_Roll!$C$21</f>
+        <f>(DCF!$E$10/(1+$B7)^0.5+DCF!$F$10/(1+$B7)^1.5+DCF!$G$10/(1+$B7)^2.5+DCF!$H$10/(1+$B7)^3.5+DCF!$I$10/(1+$B7)^4.5+DCF!$I$10*(1+D$5)/($B7-D$5)/(1+$B7)^4.5+DCF!$D$24)/Equity_Roll!$C$21</f>
         <v/>
       </c>
       <c r="E7" s="14">
-        <f>(DCF!$E$10/(1+$B7)^0.5+DCF!$F$10/(1+$B7)^1.5+DCF!$G$10/(1+$B7)^2.5+DCF!$H$10/(1+$B7)^3.5+DCF!$I$10/(1+$B7)^4.5+DCF!$I$10*(1+E$5)/($B7-E$5)/(1+$B7)^4.5+DCF!$D$23)/Equity_Roll!$C$21</f>
+        <f>(DCF!$E$10/(1+$B7)^0.5+DCF!$F$10/(1+$B7)^1.5+DCF!$G$10/(1+$B7)^2.5+DCF!$H$10/(1+$B7)^3.5+DCF!$I$10/(1+$B7)^4.5+DCF!$I$10*(1+E$5)/($B7-E$5)/(1+$B7)^4.5+DCF!$D$24)/Equity_Roll!$C$21</f>
         <v/>
       </c>
       <c r="F7" s="14">
-        <f>(DCF!$E$10/(1+$B7)^0.5+DCF!$F$10/(1+$B7)^1.5+DCF!$G$10/(1+$B7)^2.5+DCF!$H$10/(1+$B7)^3.5+DCF!$I$10/(1+$B7)^4.5+DCF!$I$10*(1+F$5)/($B7-F$5)/(1+$B7)^4.5+DCF!$D$23)/Equity_Roll!$C$21</f>
+        <f>(DCF!$E$10/(1+$B7)^0.5+DCF!$F$10/(1+$B7)^1.5+DCF!$G$10/(1+$B7)^2.5+DCF!$H$10/(1+$B7)^3.5+DCF!$I$10/(1+$B7)^4.5+DCF!$I$10*(1+F$5)/($B7-F$5)/(1+$B7)^4.5+DCF!$D$24)/Equity_Roll!$C$21</f>
         <v/>
       </c>
       <c r="G7" s="14">
-        <f>(DCF!$E$10/(1+$B7)^0.5+DCF!$F$10/(1+$B7)^1.5+DCF!$G$10/(1+$B7)^2.5+DCF!$H$10/(1+$B7)^3.5+DCF!$I$10/(1+$B7)^4.5+DCF!$I$10*(1+G$5)/($B7-G$5)/(1+$B7)^4.5+DCF!$D$23)/Equity_Roll!$C$21</f>
+        <f>(DCF!$E$10/(1+$B7)^0.5+DCF!$F$10/(1+$B7)^1.5+DCF!$G$10/(1+$B7)^2.5+DCF!$H$10/(1+$B7)^3.5+DCF!$I$10/(1+$B7)^4.5+DCF!$I$10*(1+G$5)/($B7-G$5)/(1+$B7)^4.5+DCF!$D$24)/Equity_Roll!$C$21</f>
         <v/>
       </c>
     </row>
@@ -7016,23 +7080,23 @@
         <v/>
       </c>
       <c r="C8" s="14">
-        <f>(DCF!$E$10/(1+$B8)^0.5+DCF!$F$10/(1+$B8)^1.5+DCF!$G$10/(1+$B8)^2.5+DCF!$H$10/(1+$B8)^3.5+DCF!$I$10/(1+$B8)^4.5+DCF!$I$10*(1+C$5)/($B8-C$5)/(1+$B8)^4.5+DCF!$D$23)/Equity_Roll!$C$21</f>
+        <f>(DCF!$E$10/(1+$B8)^0.5+DCF!$F$10/(1+$B8)^1.5+DCF!$G$10/(1+$B8)^2.5+DCF!$H$10/(1+$B8)^3.5+DCF!$I$10/(1+$B8)^4.5+DCF!$I$10*(1+C$5)/($B8-C$5)/(1+$B8)^4.5+DCF!$D$24)/Equity_Roll!$C$21</f>
         <v/>
       </c>
       <c r="D8" s="14">
-        <f>(DCF!$E$10/(1+$B8)^0.5+DCF!$F$10/(1+$B8)^1.5+DCF!$G$10/(1+$B8)^2.5+DCF!$H$10/(1+$B8)^3.5+DCF!$I$10/(1+$B8)^4.5+DCF!$I$10*(1+D$5)/($B8-D$5)/(1+$B8)^4.5+DCF!$D$23)/Equity_Roll!$C$21</f>
+        <f>(DCF!$E$10/(1+$B8)^0.5+DCF!$F$10/(1+$B8)^1.5+DCF!$G$10/(1+$B8)^2.5+DCF!$H$10/(1+$B8)^3.5+DCF!$I$10/(1+$B8)^4.5+DCF!$I$10*(1+D$5)/($B8-D$5)/(1+$B8)^4.5+DCF!$D$24)/Equity_Roll!$C$21</f>
         <v/>
       </c>
       <c r="E8" s="49">
-        <f>(DCF!$E$10/(1+$B8)^0.5+DCF!$F$10/(1+$B8)^1.5+DCF!$G$10/(1+$B8)^2.5+DCF!$H$10/(1+$B8)^3.5+DCF!$I$10/(1+$B8)^4.5+DCF!$I$10*(1+E$5)/($B8-E$5)/(1+$B8)^4.5+DCF!$D$23)/Equity_Roll!$C$21</f>
+        <f>(DCF!$E$10/(1+$B8)^0.5+DCF!$F$10/(1+$B8)^1.5+DCF!$G$10/(1+$B8)^2.5+DCF!$H$10/(1+$B8)^3.5+DCF!$I$10/(1+$B8)^4.5+DCF!$I$10*(1+E$5)/($B8-E$5)/(1+$B8)^4.5+DCF!$D$24)/Equity_Roll!$C$21</f>
         <v/>
       </c>
       <c r="F8" s="14">
-        <f>(DCF!$E$10/(1+$B8)^0.5+DCF!$F$10/(1+$B8)^1.5+DCF!$G$10/(1+$B8)^2.5+DCF!$H$10/(1+$B8)^3.5+DCF!$I$10/(1+$B8)^4.5+DCF!$I$10*(1+F$5)/($B8-F$5)/(1+$B8)^4.5+DCF!$D$23)/Equity_Roll!$C$21</f>
+        <f>(DCF!$E$10/(1+$B8)^0.5+DCF!$F$10/(1+$B8)^1.5+DCF!$G$10/(1+$B8)^2.5+DCF!$H$10/(1+$B8)^3.5+DCF!$I$10/(1+$B8)^4.5+DCF!$I$10*(1+F$5)/($B8-F$5)/(1+$B8)^4.5+DCF!$D$24)/Equity_Roll!$C$21</f>
         <v/>
       </c>
       <c r="G8" s="14">
-        <f>(DCF!$E$10/(1+$B8)^0.5+DCF!$F$10/(1+$B8)^1.5+DCF!$G$10/(1+$B8)^2.5+DCF!$H$10/(1+$B8)^3.5+DCF!$I$10/(1+$B8)^4.5+DCF!$I$10*(1+G$5)/($B8-G$5)/(1+$B8)^4.5+DCF!$D$23)/Equity_Roll!$C$21</f>
+        <f>(DCF!$E$10/(1+$B8)^0.5+DCF!$F$10/(1+$B8)^1.5+DCF!$G$10/(1+$B8)^2.5+DCF!$H$10/(1+$B8)^3.5+DCF!$I$10/(1+$B8)^4.5+DCF!$I$10*(1+G$5)/($B8-G$5)/(1+$B8)^4.5+DCF!$D$24)/Equity_Roll!$C$21</f>
         <v/>
       </c>
     </row>
@@ -7042,23 +7106,23 @@
         <v/>
       </c>
       <c r="C9" s="14">
-        <f>(DCF!$E$10/(1+$B9)^0.5+DCF!$F$10/(1+$B9)^1.5+DCF!$G$10/(1+$B9)^2.5+DCF!$H$10/(1+$B9)^3.5+DCF!$I$10/(1+$B9)^4.5+DCF!$I$10*(1+C$5)/($B9-C$5)/(1+$B9)^4.5+DCF!$D$23)/Equity_Roll!$C$21</f>
+        <f>(DCF!$E$10/(1+$B9)^0.5+DCF!$F$10/(1+$B9)^1.5+DCF!$G$10/(1+$B9)^2.5+DCF!$H$10/(1+$B9)^3.5+DCF!$I$10/(1+$B9)^4.5+DCF!$I$10*(1+C$5)/($B9-C$5)/(1+$B9)^4.5+DCF!$D$24)/Equity_Roll!$C$21</f>
         <v/>
       </c>
       <c r="D9" s="14">
-        <f>(DCF!$E$10/(1+$B9)^0.5+DCF!$F$10/(1+$B9)^1.5+DCF!$G$10/(1+$B9)^2.5+DCF!$H$10/(1+$B9)^3.5+DCF!$I$10/(1+$B9)^4.5+DCF!$I$10*(1+D$5)/($B9-D$5)/(1+$B9)^4.5+DCF!$D$23)/Equity_Roll!$C$21</f>
+        <f>(DCF!$E$10/(1+$B9)^0.5+DCF!$F$10/(1+$B9)^1.5+DCF!$G$10/(1+$B9)^2.5+DCF!$H$10/(1+$B9)^3.5+DCF!$I$10/(1+$B9)^4.5+DCF!$I$10*(1+D$5)/($B9-D$5)/(1+$B9)^4.5+DCF!$D$24)/Equity_Roll!$C$21</f>
         <v/>
       </c>
       <c r="E9" s="14">
-        <f>(DCF!$E$10/(1+$B9)^0.5+DCF!$F$10/(1+$B9)^1.5+DCF!$G$10/(1+$B9)^2.5+DCF!$H$10/(1+$B9)^3.5+DCF!$I$10/(1+$B9)^4.5+DCF!$I$10*(1+E$5)/($B9-E$5)/(1+$B9)^4.5+DCF!$D$23)/Equity_Roll!$C$21</f>
+        <f>(DCF!$E$10/(1+$B9)^0.5+DCF!$F$10/(1+$B9)^1.5+DCF!$G$10/(1+$B9)^2.5+DCF!$H$10/(1+$B9)^3.5+DCF!$I$10/(1+$B9)^4.5+DCF!$I$10*(1+E$5)/($B9-E$5)/(1+$B9)^4.5+DCF!$D$24)/Equity_Roll!$C$21</f>
         <v/>
       </c>
       <c r="F9" s="14">
-        <f>(DCF!$E$10/(1+$B9)^0.5+DCF!$F$10/(1+$B9)^1.5+DCF!$G$10/(1+$B9)^2.5+DCF!$H$10/(1+$B9)^3.5+DCF!$I$10/(1+$B9)^4.5+DCF!$I$10*(1+F$5)/($B9-F$5)/(1+$B9)^4.5+DCF!$D$23)/Equity_Roll!$C$21</f>
+        <f>(DCF!$E$10/(1+$B9)^0.5+DCF!$F$10/(1+$B9)^1.5+DCF!$G$10/(1+$B9)^2.5+DCF!$H$10/(1+$B9)^3.5+DCF!$I$10/(1+$B9)^4.5+DCF!$I$10*(1+F$5)/($B9-F$5)/(1+$B9)^4.5+DCF!$D$24)/Equity_Roll!$C$21</f>
         <v/>
       </c>
       <c r="G9" s="14">
-        <f>(DCF!$E$10/(1+$B9)^0.5+DCF!$F$10/(1+$B9)^1.5+DCF!$G$10/(1+$B9)^2.5+DCF!$H$10/(1+$B9)^3.5+DCF!$I$10/(1+$B9)^4.5+DCF!$I$10*(1+G$5)/($B9-G$5)/(1+$B9)^4.5+DCF!$D$23)/Equity_Roll!$C$21</f>
+        <f>(DCF!$E$10/(1+$B9)^0.5+DCF!$F$10/(1+$B9)^1.5+DCF!$G$10/(1+$B9)^2.5+DCF!$H$10/(1+$B9)^3.5+DCF!$I$10/(1+$B9)^4.5+DCF!$I$10*(1+G$5)/($B9-G$5)/(1+$B9)^4.5+DCF!$D$24)/Equity_Roll!$C$21</f>
         <v/>
       </c>
     </row>
@@ -7068,23 +7132,23 @@
         <v/>
       </c>
       <c r="C10" s="14">
-        <f>(DCF!$E$10/(1+$B10)^0.5+DCF!$F$10/(1+$B10)^1.5+DCF!$G$10/(1+$B10)^2.5+DCF!$H$10/(1+$B10)^3.5+DCF!$I$10/(1+$B10)^4.5+DCF!$I$10*(1+C$5)/($B10-C$5)/(1+$B10)^4.5+DCF!$D$23)/Equity_Roll!$C$21</f>
+        <f>(DCF!$E$10/(1+$B10)^0.5+DCF!$F$10/(1+$B10)^1.5+DCF!$G$10/(1+$B10)^2.5+DCF!$H$10/(1+$B10)^3.5+DCF!$I$10/(1+$B10)^4.5+DCF!$I$10*(1+C$5)/($B10-C$5)/(1+$B10)^4.5+DCF!$D$24)/Equity_Roll!$C$21</f>
         <v/>
       </c>
       <c r="D10" s="14">
-        <f>(DCF!$E$10/(1+$B10)^0.5+DCF!$F$10/(1+$B10)^1.5+DCF!$G$10/(1+$B10)^2.5+DCF!$H$10/(1+$B10)^3.5+DCF!$I$10/(1+$B10)^4.5+DCF!$I$10*(1+D$5)/($B10-D$5)/(1+$B10)^4.5+DCF!$D$23)/Equity_Roll!$C$21</f>
+        <f>(DCF!$E$10/(1+$B10)^0.5+DCF!$F$10/(1+$B10)^1.5+DCF!$G$10/(1+$B10)^2.5+DCF!$H$10/(1+$B10)^3.5+DCF!$I$10/(1+$B10)^4.5+DCF!$I$10*(1+D$5)/($B10-D$5)/(1+$B10)^4.5+DCF!$D$24)/Equity_Roll!$C$21</f>
         <v/>
       </c>
       <c r="E10" s="14">
-        <f>(DCF!$E$10/(1+$B10)^0.5+DCF!$F$10/(1+$B10)^1.5+DCF!$G$10/(1+$B10)^2.5+DCF!$H$10/(1+$B10)^3.5+DCF!$I$10/(1+$B10)^4.5+DCF!$I$10*(1+E$5)/($B10-E$5)/(1+$B10)^4.5+DCF!$D$23)/Equity_Roll!$C$21</f>
+        <f>(DCF!$E$10/(1+$B10)^0.5+DCF!$F$10/(1+$B10)^1.5+DCF!$G$10/(1+$B10)^2.5+DCF!$H$10/(1+$B10)^3.5+DCF!$I$10/(1+$B10)^4.5+DCF!$I$10*(1+E$5)/($B10-E$5)/(1+$B10)^4.5+DCF!$D$24)/Equity_Roll!$C$21</f>
         <v/>
       </c>
       <c r="F10" s="14">
-        <f>(DCF!$E$10/(1+$B10)^0.5+DCF!$F$10/(1+$B10)^1.5+DCF!$G$10/(1+$B10)^2.5+DCF!$H$10/(1+$B10)^3.5+DCF!$I$10/(1+$B10)^4.5+DCF!$I$10*(1+F$5)/($B10-F$5)/(1+$B10)^4.5+DCF!$D$23)/Equity_Roll!$C$21</f>
+        <f>(DCF!$E$10/(1+$B10)^0.5+DCF!$F$10/(1+$B10)^1.5+DCF!$G$10/(1+$B10)^2.5+DCF!$H$10/(1+$B10)^3.5+DCF!$I$10/(1+$B10)^4.5+DCF!$I$10*(1+F$5)/($B10-F$5)/(1+$B10)^4.5+DCF!$D$24)/Equity_Roll!$C$21</f>
         <v/>
       </c>
       <c r="G10" s="14">
-        <f>(DCF!$E$10/(1+$B10)^0.5+DCF!$F$10/(1+$B10)^1.5+DCF!$G$10/(1+$B10)^2.5+DCF!$H$10/(1+$B10)^3.5+DCF!$I$10/(1+$B10)^4.5+DCF!$I$10*(1+G$5)/($B10-G$5)/(1+$B10)^4.5+DCF!$D$23)/Equity_Roll!$C$21</f>
+        <f>(DCF!$E$10/(1+$B10)^0.5+DCF!$F$10/(1+$B10)^1.5+DCF!$G$10/(1+$B10)^2.5+DCF!$H$10/(1+$B10)^3.5+DCF!$I$10/(1+$B10)^4.5+DCF!$I$10*(1+G$5)/($B10-G$5)/(1+$B10)^4.5+DCF!$D$24)/Equity_Roll!$C$21</f>
         <v/>
       </c>
     </row>
@@ -7313,11 +7377,11 @@
         <v>-40</v>
       </c>
       <c r="C24" s="14">
-        <f>((DCF!E$10+$B24/365*(IS!E$6-IS!D$6))/(1+Assumptions!$C$86)^0.5+(DCF!F$10+$B24/365*(IS!F$6-IS!E$6))/(1+Assumptions!$C$86)^1.5+(DCF!G$10+$B24/365*(IS!G$6-IS!F$6))/(1+Assumptions!$C$86)^2.5+(DCF!H$10+$B24/365*(IS!H$6-IS!G$6))/(1+Assumptions!$C$86)^3.5+(DCF!I$10+$B24/365*(IS!I$6-IS!H$6))/(1+Assumptions!$C$86)^4.5+(DCF!$I$10+$B24/365*(IS!I$6-IS!H$6))*(1+Assumptions!$C$87)/(Assumptions!$C$86-Assumptions!$C$87)/(1+Assumptions!$C$86)^4.5+DCF!$D$23)/Equity_Roll!$C$21</f>
+        <f>((DCF!E$10+$B24/365*(IS!E$6-IS!D$6))/(1+Assumptions!$C$86)^0.5+(DCF!F$10+$B24/365*(IS!F$6-IS!E$6))/(1+Assumptions!$C$86)^1.5+(DCF!G$10+$B24/365*(IS!G$6-IS!F$6))/(1+Assumptions!$C$86)^2.5+(DCF!H$10+$B24/365*(IS!H$6-IS!G$6))/(1+Assumptions!$C$86)^3.5+(DCF!I$10+$B24/365*(IS!I$6-IS!H$6))/(1+Assumptions!$C$86)^4.5+(DCF!$I$10+$B24/365*(IS!I$6-IS!H$6))*(1+Assumptions!$C$87)/(Assumptions!$C$86-Assumptions!$C$87)/(1+Assumptions!$C$86)^4.5+DCF!$D$24)/Equity_Roll!$C$21</f>
         <v/>
       </c>
       <c r="D24" s="16">
-        <f>C24/DCF!$D$25-1</f>
+        <f>C24/DCF!$D$26-1</f>
         <v/>
       </c>
     </row>
@@ -7326,11 +7390,11 @@
         <v>-20</v>
       </c>
       <c r="C25" s="14">
-        <f>((DCF!E$10+$B25/365*(IS!E$6-IS!D$6))/(1+Assumptions!$C$86)^0.5+(DCF!F$10+$B25/365*(IS!F$6-IS!E$6))/(1+Assumptions!$C$86)^1.5+(DCF!G$10+$B25/365*(IS!G$6-IS!F$6))/(1+Assumptions!$C$86)^2.5+(DCF!H$10+$B25/365*(IS!H$6-IS!G$6))/(1+Assumptions!$C$86)^3.5+(DCF!I$10+$B25/365*(IS!I$6-IS!H$6))/(1+Assumptions!$C$86)^4.5+(DCF!$I$10+$B25/365*(IS!I$6-IS!H$6))*(1+Assumptions!$C$87)/(Assumptions!$C$86-Assumptions!$C$87)/(1+Assumptions!$C$86)^4.5+DCF!$D$23)/Equity_Roll!$C$21</f>
+        <f>((DCF!E$10+$B25/365*(IS!E$6-IS!D$6))/(1+Assumptions!$C$86)^0.5+(DCF!F$10+$B25/365*(IS!F$6-IS!E$6))/(1+Assumptions!$C$86)^1.5+(DCF!G$10+$B25/365*(IS!G$6-IS!F$6))/(1+Assumptions!$C$86)^2.5+(DCF!H$10+$B25/365*(IS!H$6-IS!G$6))/(1+Assumptions!$C$86)^3.5+(DCF!I$10+$B25/365*(IS!I$6-IS!H$6))/(1+Assumptions!$C$86)^4.5+(DCF!$I$10+$B25/365*(IS!I$6-IS!H$6))*(1+Assumptions!$C$87)/(Assumptions!$C$86-Assumptions!$C$87)/(1+Assumptions!$C$86)^4.5+DCF!$D$24)/Equity_Roll!$C$21</f>
         <v/>
       </c>
       <c r="D25" s="16">
-        <f>C25/DCF!$D$25-1</f>
+        <f>C25/DCF!$D$26-1</f>
         <v/>
       </c>
     </row>
@@ -7339,11 +7403,11 @@
         <v>0</v>
       </c>
       <c r="C26" s="49">
-        <f>((DCF!E$10+$B26/365*(IS!E$6-IS!D$6))/(1+Assumptions!$C$86)^0.5+(DCF!F$10+$B26/365*(IS!F$6-IS!E$6))/(1+Assumptions!$C$86)^1.5+(DCF!G$10+$B26/365*(IS!G$6-IS!F$6))/(1+Assumptions!$C$86)^2.5+(DCF!H$10+$B26/365*(IS!H$6-IS!G$6))/(1+Assumptions!$C$86)^3.5+(DCF!I$10+$B26/365*(IS!I$6-IS!H$6))/(1+Assumptions!$C$86)^4.5+(DCF!$I$10+$B26/365*(IS!I$6-IS!H$6))*(1+Assumptions!$C$87)/(Assumptions!$C$86-Assumptions!$C$87)/(1+Assumptions!$C$86)^4.5+DCF!$D$23)/Equity_Roll!$C$21</f>
+        <f>((DCF!E$10+$B26/365*(IS!E$6-IS!D$6))/(1+Assumptions!$C$86)^0.5+(DCF!F$10+$B26/365*(IS!F$6-IS!E$6))/(1+Assumptions!$C$86)^1.5+(DCF!G$10+$B26/365*(IS!G$6-IS!F$6))/(1+Assumptions!$C$86)^2.5+(DCF!H$10+$B26/365*(IS!H$6-IS!G$6))/(1+Assumptions!$C$86)^3.5+(DCF!I$10+$B26/365*(IS!I$6-IS!H$6))/(1+Assumptions!$C$86)^4.5+(DCF!$I$10+$B26/365*(IS!I$6-IS!H$6))*(1+Assumptions!$C$87)/(Assumptions!$C$86-Assumptions!$C$87)/(1+Assumptions!$C$86)^4.5+DCF!$D$24)/Equity_Roll!$C$21</f>
         <v/>
       </c>
       <c r="D26" s="16">
-        <f>C26/DCF!$D$25-1</f>
+        <f>C26/DCF!$D$26-1</f>
         <v/>
       </c>
     </row>
@@ -7352,11 +7416,11 @@
         <v>20</v>
       </c>
       <c r="C27" s="14">
-        <f>((DCF!E$10+$B27/365*(IS!E$6-IS!D$6))/(1+Assumptions!$C$86)^0.5+(DCF!F$10+$B27/365*(IS!F$6-IS!E$6))/(1+Assumptions!$C$86)^1.5+(DCF!G$10+$B27/365*(IS!G$6-IS!F$6))/(1+Assumptions!$C$86)^2.5+(DCF!H$10+$B27/365*(IS!H$6-IS!G$6))/(1+Assumptions!$C$86)^3.5+(DCF!I$10+$B27/365*(IS!I$6-IS!H$6))/(1+Assumptions!$C$86)^4.5+(DCF!$I$10+$B27/365*(IS!I$6-IS!H$6))*(1+Assumptions!$C$87)/(Assumptions!$C$86-Assumptions!$C$87)/(1+Assumptions!$C$86)^4.5+DCF!$D$23)/Equity_Roll!$C$21</f>
+        <f>((DCF!E$10+$B27/365*(IS!E$6-IS!D$6))/(1+Assumptions!$C$86)^0.5+(DCF!F$10+$B27/365*(IS!F$6-IS!E$6))/(1+Assumptions!$C$86)^1.5+(DCF!G$10+$B27/365*(IS!G$6-IS!F$6))/(1+Assumptions!$C$86)^2.5+(DCF!H$10+$B27/365*(IS!H$6-IS!G$6))/(1+Assumptions!$C$86)^3.5+(DCF!I$10+$B27/365*(IS!I$6-IS!H$6))/(1+Assumptions!$C$86)^4.5+(DCF!$I$10+$B27/365*(IS!I$6-IS!H$6))*(1+Assumptions!$C$87)/(Assumptions!$C$86-Assumptions!$C$87)/(1+Assumptions!$C$86)^4.5+DCF!$D$24)/Equity_Roll!$C$21</f>
         <v/>
       </c>
       <c r="D27" s="16">
-        <f>C27/DCF!$D$25-1</f>
+        <f>C27/DCF!$D$26-1</f>
         <v/>
       </c>
     </row>
@@ -7365,11 +7429,11 @@
         <v>40</v>
       </c>
       <c r="C28" s="14">
-        <f>((DCF!E$10+$B28/365*(IS!E$6-IS!D$6))/(1+Assumptions!$C$86)^0.5+(DCF!F$10+$B28/365*(IS!F$6-IS!E$6))/(1+Assumptions!$C$86)^1.5+(DCF!G$10+$B28/365*(IS!G$6-IS!F$6))/(1+Assumptions!$C$86)^2.5+(DCF!H$10+$B28/365*(IS!H$6-IS!G$6))/(1+Assumptions!$C$86)^3.5+(DCF!I$10+$B28/365*(IS!I$6-IS!H$6))/(1+Assumptions!$C$86)^4.5+(DCF!$I$10+$B28/365*(IS!I$6-IS!H$6))*(1+Assumptions!$C$87)/(Assumptions!$C$86-Assumptions!$C$87)/(1+Assumptions!$C$86)^4.5+DCF!$D$23)/Equity_Roll!$C$21</f>
+        <f>((DCF!E$10+$B28/365*(IS!E$6-IS!D$6))/(1+Assumptions!$C$86)^0.5+(DCF!F$10+$B28/365*(IS!F$6-IS!E$6))/(1+Assumptions!$C$86)^1.5+(DCF!G$10+$B28/365*(IS!G$6-IS!F$6))/(1+Assumptions!$C$86)^2.5+(DCF!H$10+$B28/365*(IS!H$6-IS!G$6))/(1+Assumptions!$C$86)^3.5+(DCF!I$10+$B28/365*(IS!I$6-IS!H$6))/(1+Assumptions!$C$86)^4.5+(DCF!$I$10+$B28/365*(IS!I$6-IS!H$6))*(1+Assumptions!$C$87)/(Assumptions!$C$86-Assumptions!$C$87)/(1+Assumptions!$C$86)^4.5+DCF!$D$24)/Equity_Roll!$C$21</f>
         <v/>
       </c>
       <c r="D28" s="16">
-        <f>C28/DCF!$D$25-1</f>
+        <f>C28/DCF!$D$26-1</f>
         <v/>
       </c>
     </row>
@@ -7617,7 +7681,7 @@
         </is>
       </c>
       <c r="B12" s="17">
-        <f>(E11/(1+Assumptions!$C$86)^0.5+F11/(1+Assumptions!$C$86)^1.5+G11/(1+Assumptions!$C$86)^2.5+H11/(1+Assumptions!$C$86)^3.5+I11/(1+Assumptions!$C$86)^4.5+I11*(1+Assumptions!$C$87)/(Assumptions!$C$86-Assumptions!$C$87)/(1+Assumptions!$C$86)^4.5+DCF!$D$23)/Equity_Roll!$C$21</f>
+        <f>(E11/(1+Assumptions!$C$86)^0.5+F11/(1+Assumptions!$C$86)^1.5+G11/(1+Assumptions!$C$86)^2.5+H11/(1+Assumptions!$C$86)^3.5+I11/(1+Assumptions!$C$86)^4.5+I11*(1+Assumptions!$C$87)/(Assumptions!$C$86-Assumptions!$C$87)/(1+Assumptions!$C$86)^4.5+DCF!$D$24)/Equity_Roll!$C$21</f>
         <v/>
       </c>
       <c r="J12" s="11" t="inlineStr">
@@ -7796,7 +7860,7 @@
         </is>
       </c>
       <c r="B21" s="17">
-        <f>DCF!D25</f>
+        <f>DCF!D26</f>
         <v/>
       </c>
       <c r="J21" s="11" t="inlineStr">
@@ -7982,7 +8046,7 @@
         </is>
       </c>
       <c r="B31" s="17">
-        <f>(E30/(1+Assumptions!$C$86)^0.5+F30/(1+Assumptions!$C$86)^1.5+G30/(1+Assumptions!$C$86)^2.5+H30/(1+Assumptions!$C$86)^3.5+I30/(1+Assumptions!$C$86)^4.5+I30*(1+Assumptions!$C$87)/(Assumptions!$C$86-Assumptions!$C$87)/(1+Assumptions!$C$86)^4.5+DCF!$D$23)/Equity_Roll!$C$21</f>
+        <f>(E30/(1+Assumptions!$C$86)^0.5+F30/(1+Assumptions!$C$86)^1.5+G30/(1+Assumptions!$C$86)^2.5+H30/(1+Assumptions!$C$86)^3.5+I30/(1+Assumptions!$C$86)^4.5+I30*(1+Assumptions!$C$87)/(Assumptions!$C$86-Assumptions!$C$87)/(1+Assumptions!$C$86)^4.5+DCF!$D$24)/Equity_Roll!$C$21</f>
         <v/>
       </c>
       <c r="J31" s="11" t="inlineStr">
@@ -8433,7 +8497,7 @@
         </is>
       </c>
       <c r="B9" s="54">
-        <f>DCF!D25&gt;0</f>
+        <f>DCF!D26&gt;0</f>
         <v/>
       </c>
       <c r="J9" s="11" t="inlineStr">
@@ -8449,7 +8513,7 @@
         </is>
       </c>
       <c r="B10" s="54">
-        <f>ABS(Sensitivity!E8-DCF!D25)&lt;0.01</f>
+        <f>ABS(Sensitivity!E8-DCF!D26)&lt;0.01</f>
         <v/>
       </c>
       <c r="J10" s="11" t="inlineStr">
@@ -8672,11 +8736,11 @@
         </is>
       </c>
       <c r="B21" s="16">
-        <f>FCFE!D18/DCF!D25</f>
+        <f>FCFE!D20/DCF!D26</f>
         <v/>
       </c>
       <c r="C21" s="14">
-        <f>FCFE!D18</f>
+        <f>FCFE!D20</f>
         <v/>
       </c>
       <c r="J21" s="11" t="inlineStr">
@@ -8819,11 +8883,11 @@
         </is>
       </c>
       <c r="C5" s="14">
-        <f>DCF!D25</f>
+        <f>DCF!D26</f>
         <v/>
       </c>
       <c r="D5" s="14">
-        <f>DCF!D25</f>
+        <f>DCF!D26</f>
         <v/>
       </c>
       <c r="E5" s="15">
@@ -8984,11 +9048,11 @@
         </is>
       </c>
       <c r="C10" s="14">
-        <f>FCFE!D18</f>
+        <f>FCFE!D20</f>
         <v/>
       </c>
       <c r="D10" s="14">
-        <f>FCFE!D18</f>
+        <f>FCFE!D20</f>
         <v/>
       </c>
       <c r="E10" s="15">

</xml_diff>